<commit_message>
Temps en texte mm:ss (sans millisecondes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SjSsUvYfWg3LPV8sLWWofN
</commit_message>
<xml_diff>
--- a/Classement_1.xlsx
+++ b/Classement_1.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -78,6 +78,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -522,8 +525,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>0.005995370370370371</v>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>8:38</t>
+        </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -558,8 +563,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>0.006122685185185185</v>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>8:49</t>
+        </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -594,8 +601,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>0.006168981481481482</v>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>8:53</t>
+        </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -630,8 +639,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>0.006481481481481481</v>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>9:20</t>
+        </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -666,8 +677,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>0.006712962962962963</v>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -702,8 +715,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>0.006724537037037037</v>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>9:41</t>
+        </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -738,8 +753,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n">
-        <v>0.006886574074074074</v>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>9:55</t>
+        </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -774,8 +791,10 @@
           <t>2nd PRO GAIA</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>0.006898148148148148</v>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>9:56</t>
+        </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -810,8 +829,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n">
-        <v>0.006909722222222222</v>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>9:57</t>
+        </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -846,8 +867,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>0.006956018518518518</v>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -882,8 +905,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>0.006990740740740741</v>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -918,8 +943,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>0.007083333333333333</v>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -954,8 +981,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>0.007175925925925926</v>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -990,8 +1019,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>0.007222222222222222</v>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1026,8 +1057,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n">
-        <v>0.007233796296296296</v>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1062,8 +1095,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n">
-        <v>0.007256944444444444</v>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1098,8 +1133,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n">
-        <v>0.00730324074074074</v>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1134,8 +1171,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n">
-        <v>0.007337962962962963</v>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1170,8 +1209,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>0.007372685185185185</v>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>10:37</t>
+        </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1206,8 +1247,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n">
-        <v>0.007430555555555556</v>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -1242,8 +1285,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>0.007465277777777778</v>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1278,8 +1323,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n">
-        <v>0.007476851851851852</v>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>10:46</t>
+        </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -1314,8 +1361,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n">
-        <v>0.007488425925925926</v>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1350,8 +1399,10 @@
           <t>Prof</t>
         </is>
       </c>
-      <c r="F25" s="4" t="n">
-        <v>0.0075</v>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -1382,8 +1433,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F26" s="4" t="n">
-        <v>0.0075</v>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -1418,8 +1471,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F27" s="4" t="n">
-        <v>0.007523148148148148</v>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -1454,8 +1509,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F28" s="4" t="n">
-        <v>0.007534722222222222</v>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>10:51</t>
+        </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -1490,8 +1547,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F29" s="4" t="n">
-        <v>0.00755787037037037</v>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -1526,8 +1585,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F30" s="4" t="n">
-        <v>0.007569444444444445</v>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -1562,8 +1623,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F31" s="4" t="n">
-        <v>0.007592592592592593</v>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -1598,8 +1661,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F32" s="4" t="n">
-        <v>0.007650462962962963</v>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -1634,8 +1699,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F33" s="4" t="n">
-        <v>0.007696759259259259</v>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -1670,8 +1737,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F34" s="4" t="n">
-        <v>0.007708333333333334</v>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
@@ -1706,8 +1775,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F35" s="4" t="n">
-        <v>0.007708333333333334</v>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -1742,8 +1813,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F36" s="4" t="n">
-        <v>0.007731481481481482</v>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -1778,8 +1851,10 @@
           <t>1ere PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F37" s="4" t="n">
-        <v>0.007766203703703704</v>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -1814,8 +1889,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F38" s="4" t="n">
-        <v>0.007800925925925926</v>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>11:14</t>
+        </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -1850,8 +1927,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F39" s="4" t="n">
-        <v>0.008078703703703704</v>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -1886,8 +1965,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F40" s="4" t="n">
-        <v>0.008101851851851851</v>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -1922,8 +2003,10 @@
           <t>2nd Pro PASTEUR</t>
         </is>
       </c>
-      <c r="F41" s="4" t="n">
-        <v>0.008171296296296296</v>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -1958,8 +2041,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F42" s="4" t="n">
-        <v>0.008252314814814815</v>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -1994,8 +2079,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F43" s="4" t="n">
-        <v>0.008287037037037037</v>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -2030,8 +2117,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F44" s="4" t="n">
-        <v>0.00832175925925926</v>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>11:59</t>
+        </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -2066,8 +2155,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F45" s="4" t="n">
-        <v>0.008333333333333333</v>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -2102,8 +2193,10 @@
           <t>Prof</t>
         </is>
       </c>
-      <c r="F46" s="4" t="n">
-        <v>0.008356481481481482</v>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -2134,8 +2227,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F47" s="4" t="n">
-        <v>0.008402777777777778</v>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>12:06</t>
+        </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -2170,8 +2265,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F48" s="4" t="n">
-        <v>0.00849537037037037</v>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -2206,8 +2303,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F49" s="4" t="n">
-        <v>0.008564814814814815</v>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -2242,8 +2341,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F50" s="4" t="n">
-        <v>0.008576388888888889</v>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -2278,8 +2379,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F51" s="4" t="n">
-        <v>0.008668981481481481</v>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>12:29</t>
+        </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -2314,8 +2417,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F52" s="4" t="n">
-        <v>0.008726851851851852</v>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -2350,8 +2455,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F53" s="4" t="n">
-        <v>0.008773148148148148</v>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -2386,8 +2493,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F54" s="4" t="n">
-        <v>0.008819444444444444</v>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
@@ -2422,8 +2531,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F55" s="4" t="n">
-        <v>0.008900462962962962</v>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
@@ -2458,8 +2569,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F56" s="4" t="n">
-        <v>0.009027777777777777</v>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -2494,8 +2607,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F57" s="4" t="n">
-        <v>0.009074074074074075</v>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -2530,8 +2645,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F58" s="4" t="n">
-        <v>0.009189814814814816</v>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -2566,8 +2683,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F59" s="4" t="n">
-        <v>0.009212962962962963</v>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>13:16</t>
+        </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -2602,8 +2721,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F60" s="4" t="n">
-        <v>0.009224537037037036</v>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -2638,8 +2759,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F61" s="4" t="n">
-        <v>0.00931712962962963</v>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -2674,8 +2797,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F62" s="4" t="n">
-        <v>0.009328703703703704</v>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
@@ -2710,8 +2835,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F63" s="4" t="n">
-        <v>0.009328703703703704</v>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
@@ -2746,8 +2873,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F64" s="4" t="n">
-        <v>0.009328703703703704</v>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -2782,8 +2911,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F65" s="4" t="n">
-        <v>0.009340277777777777</v>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
@@ -2818,8 +2949,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F66" s="4" t="n">
-        <v>0.009340277777777777</v>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -2854,8 +2987,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F67" s="4" t="n">
-        <v>0.009351851851851853</v>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -2890,8 +3025,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F68" s="4" t="n">
-        <v>0.009363425925925926</v>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -2926,8 +3063,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F69" s="4" t="n">
-        <v>0.009675925925925926</v>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
@@ -2962,8 +3101,10 @@
           <t>Première Pro App</t>
         </is>
       </c>
-      <c r="F70" s="4" t="n">
-        <v>0.009699074074074074</v>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
@@ -2998,8 +3139,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F71" s="4" t="n">
-        <v>0.009699074074074074</v>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
@@ -3034,8 +3177,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F72" s="4" t="n">
-        <v>0.009699074074074074</v>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
@@ -3070,8 +3215,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F73" s="4" t="n">
-        <v>0.009699074074074074</v>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
@@ -3106,8 +3253,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F74" s="4" t="n">
-        <v>0.009710648148148149</v>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -3142,8 +3291,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F75" s="4" t="n">
-        <v>0.009710648148148149</v>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
@@ -3178,8 +3329,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F76" s="4" t="n">
-        <v>0.009710648148148149</v>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
@@ -3214,8 +3367,10 @@
           <t>Prof</t>
         </is>
       </c>
-      <c r="F77" s="4" t="n">
-        <v>0.009710648148148149</v>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
@@ -3246,8 +3401,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F78" s="4" t="n">
-        <v>0.009722222222222222</v>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
@@ -3282,8 +3439,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F79" s="4" t="n">
-        <v>0.009722222222222222</v>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
@@ -3318,8 +3477,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F80" s="4" t="n">
-        <v>0.009733796296296296</v>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
@@ -3354,8 +3515,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F81" s="4" t="n">
-        <v>0.009733796296296296</v>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
@@ -3390,8 +3553,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F82" s="4" t="n">
-        <v>0.00974537037037037</v>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
@@ -3426,8 +3591,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F83" s="4" t="n">
-        <v>0.00974537037037037</v>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
@@ -3462,8 +3629,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F84" s="4" t="n">
-        <v>0.01016203703703704</v>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
@@ -3498,8 +3667,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F85" s="4" t="n">
-        <v>0.01017361111111111</v>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>14:39</t>
+        </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
@@ -3534,8 +3705,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F86" s="4" t="n">
-        <v>0.01037037037037037</v>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
@@ -3570,8 +3743,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F87" s="4" t="n">
-        <v>0.01038194444444444</v>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
@@ -3606,8 +3781,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F88" s="4" t="n">
-        <v>0.01040509259259259</v>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
@@ -3642,8 +3819,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F89" s="4" t="n">
-        <v>0.01050925925925926</v>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
@@ -3678,8 +3857,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F90" s="4" t="n">
-        <v>0.01085648148148148</v>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
@@ -3714,8 +3895,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F91" s="4" t="n">
-        <v>0.01085648148148148</v>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
@@ -3750,8 +3933,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F92" s="4" t="n">
-        <v>0.01086805555555556</v>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
@@ -3786,8 +3971,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F93" s="4" t="n">
-        <v>0.01086805555555556</v>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
@@ -3822,8 +4009,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F94" s="4" t="n">
-        <v>0.01100694444444444</v>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
@@ -3858,8 +4047,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F95" s="4" t="n">
-        <v>0.01123842592592593</v>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
@@ -3894,8 +4085,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F96" s="4" t="n">
-        <v>0.01142361111111111</v>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
@@ -3930,8 +4123,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F97" s="4" t="n">
-        <v>0.01150462962962963</v>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
@@ -3966,8 +4161,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F98" s="4" t="n">
-        <v>0.01190972222222222</v>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
@@ -4002,8 +4199,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F99" s="4" t="n">
-        <v>0.01195601851851852</v>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>17:13</t>
+        </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
@@ -4038,8 +4237,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F100" s="4" t="n">
-        <v>0.01196759259259259</v>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
@@ -4074,8 +4275,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F101" s="4" t="n">
-        <v>0.01196759259259259</v>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
@@ -4110,8 +4313,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F102" s="4" t="n">
-        <v>0.01197916666666667</v>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
@@ -4146,8 +4351,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F103" s="4" t="n">
-        <v>0.0128587962962963</v>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
@@ -4182,8 +4389,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F104" s="4" t="n">
-        <v>0.0128587962962963</v>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
@@ -4218,8 +4427,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F105" s="4" t="n">
-        <v>0.0128587962962963</v>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
@@ -4254,8 +4465,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F106" s="4" t="n">
-        <v>0.0128587962962963</v>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
@@ -4290,8 +4503,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F107" s="4" t="n">
-        <v>0.01287037037037037</v>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
@@ -4326,8 +4541,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F108" s="4" t="n">
-        <v>0.01287037037037037</v>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
@@ -4362,8 +4579,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F109" s="4" t="n">
-        <v>0.01288194444444444</v>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
@@ -4398,8 +4617,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F110" s="4" t="n">
-        <v>0.01289351851851852</v>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
@@ -4434,8 +4655,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F111" s="4" t="n">
-        <v>0.01289351851851852</v>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
@@ -4470,8 +4693,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F112" s="4" t="n">
-        <v>0.01290509259259259</v>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
@@ -4506,8 +4731,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F113" s="4" t="n">
-        <v>0.01290509259259259</v>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
@@ -4542,8 +4769,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F114" s="4" t="n">
-        <v>0.01291666666666667</v>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
@@ -4578,8 +4807,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F115" s="4" t="n">
-        <v>0.01291666666666667</v>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
@@ -4614,8 +4845,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F116" s="4" t="n">
-        <v>0.01292824074074074</v>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
@@ -4650,8 +4883,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F117" s="4" t="n">
-        <v>0.0130787037037037</v>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
@@ -4686,8 +4921,10 @@
           <t>2nd Mendel</t>
         </is>
       </c>
-      <c r="F118" s="4" t="n">
-        <v>0.01314814814814815</v>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>18:56</t>
+        </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
@@ -4722,8 +4959,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F119" s="4" t="n">
-        <v>0.01321759259259259</v>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
@@ -4758,8 +4997,10 @@
           <t>1ere STAV</t>
         </is>
       </c>
-      <c r="F120" s="4" t="n">
-        <v>0.01321759259259259</v>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
@@ -4794,8 +5035,10 @@
           <t>2nd Pasteur</t>
         </is>
       </c>
-      <c r="F121" s="4" t="n">
-        <v>0.01321759259259259</v>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
@@ -4830,8 +5073,10 @@
           <t>Première PRO APP</t>
         </is>
       </c>
-      <c r="F122" s="4" t="n">
-        <v>0.01322916666666667</v>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>19:03</t>
+        </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
@@ -4866,8 +5111,10 @@
           <t>2nd Pro Pasteur</t>
         </is>
       </c>
-      <c r="F123" s="4" t="n">
-        <v>0.01325231481481481</v>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
@@ -4902,8 +5149,10 @@
           <t>2nd PRO ARISTEE</t>
         </is>
       </c>
-      <c r="F124" s="4" t="n">
-        <v>0.01327546296296296</v>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
@@ -4938,8 +5187,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F125" s="4" t="n">
-        <v>0.01369212962962963</v>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
@@ -4974,8 +5225,10 @@
           <t>2nd MENDEL</t>
         </is>
       </c>
-      <c r="F126" s="4" t="n">
-        <v>0.01393518518518519</v>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>20:04</t>
+        </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
@@ -5010,8 +5263,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F127" s="4" t="n">
-        <v>0.01428240740740741</v>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
@@ -5046,8 +5301,10 @@
           <t>1G</t>
         </is>
       </c>
-      <c r="F128" s="4" t="n">
-        <v>0.01430555555555556</v>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
@@ -5082,8 +5339,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F129" s="4" t="n">
-        <v>0.01430555555555556</v>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
@@ -5118,8 +5377,10 @@
           <t>Première Pro</t>
         </is>
       </c>
-      <c r="F130" s="4" t="n">
-        <v>0.01502314814814815</v>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>21:38</t>
+        </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
@@ -5154,8 +5415,10 @@
           <t>2nd Pro GAIA</t>
         </is>
       </c>
-      <c r="F131" s="4" t="n">
-        <v>0.0150462962962963</v>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>

</xml_diff>